<commit_message>
Add Spreadsheet nav link, embed logo in xlsx, add Calculator link to spreadsheet page
</commit_message>
<xml_diff>
--- a/downloads/blackcat-airbnb-profit-tracker.xlsx
+++ b/downloads/blackcat-airbnb-profit-tracker.xlsx
@@ -18,7 +18,7 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="323" uniqueCount="176">
   <si>
-    <t>🐈‍⬛ Black Cat Analytics — Airbnb Profit Tracker</t>
+    <t>Black Cat Analytics — Airbnb Profit Tracker</t>
   </si>
   <si>
     <t/>
@@ -114,7 +114,7 @@
     <t>Questions? support@tryblackcat.com</t>
   </si>
   <si>
-    <t>🐈‍⬛ Black Cat Analytics — Revenue &amp; Expense Log</t>
+    <t>Black Cat Analytics — Revenue &amp; Expense Log</t>
   </si>
   <si>
     <t>Log every Airbnb payout and expense here. The other sheets pull from this data.</t>
@@ -273,7 +273,7 @@
     <t>3% of gross</t>
   </si>
   <si>
-    <t>🐈‍⬛ Black Cat Analytics — Monthly Dashboard</t>
+    <t>Black Cat Analytics — Monthly Dashboard</t>
   </si>
   <si>
     <t>Auto-calculated from your Revenue &amp; Expenses log. Do not edit the formula cells.</t>
@@ -339,7 +339,7 @@
     <t>Avg Revenue/Transaction</t>
   </si>
   <si>
-    <t>🐈‍⬛ Black Cat Analytics — Per-Property Summary</t>
+    <t>Black Cat Analytics — Per-Property Summary</t>
   </si>
   <si>
     <t>Performance breakdown by listing. Add your property names in column A.</t>
@@ -360,7 +360,7 @@
     <t>TOTAL</t>
   </si>
   <si>
-    <t>🐈‍⬛ Black Cat Analytics — Schedule E Tax Report</t>
+    <t>Black Cat Analytics — Schedule E Tax Report</t>
   </si>
   <si>
     <t>Auto-calculated deductions mapped to IRS Schedule E line items. Adjust "Fair Rental Days" and "Personal Use Days" below.</t>
@@ -474,7 +474,7 @@
     <t>NET RENTAL INCOME (Line 21)</t>
   </si>
   <si>
-    <t>🐈‍⬛ Black Cat Analytics — Cleaning Cost Tracker</t>
+    <t>Black Cat Analytics — Cleaning Cost Tracker</t>
   </si>
   <si>
     <t>Track per-turnover cleaning costs by property. Spot overcharges and optimize your biggest variable expense.</t>
@@ -806,6 +806,226 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:oneCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="304800" cy="304800"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="1" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="0" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:oneCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="304800" cy="304800"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="1" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="0" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:oneCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="304800" cy="304800"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="1" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="0" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:oneCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="304800" cy="304800"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="1" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="0" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing5.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:oneCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="304800" cy="304800"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="1" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="0" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1337,11 +1557,10 @@
     <col min="8" max="8" width="30" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="36" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1" s="4" t="s">
+    <row r="1" ht="40" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B1" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="B1" s="4"/>
       <c r="C1" s="4"/>
       <c r="D1" s="4"/>
       <c r="E1" s="4"/>
@@ -2411,7 +2630,7 @@
     <row r="500" spans="2:7" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="B1:H1"/>
     <mergeCell ref="A2:H2"/>
   </mergeCells>
   <dataValidations count="6">
@@ -2436,6 +2655,7 @@
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -2449,11 +2669,10 @@
     <col min="14" max="14" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="36" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1" s="4" t="s">
+    <row r="1" ht="40" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B1" s="4" t="s">
         <v>85</v>
       </c>
-      <c r="B1" s="4"/>
       <c r="C1" s="4"/>
       <c r="D1" s="4"/>
       <c r="E1" s="4"/>
@@ -2784,11 +3003,12 @@
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="B1:H1"/>
     <mergeCell ref="A2:H2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -2805,11 +3025,10 @@
     <col min="8" max="8" width="22" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="36" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1" s="4" t="s">
+    <row r="1" ht="40" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B1" s="4" t="s">
         <v>107</v>
       </c>
-      <c r="B1" s="4"/>
       <c r="C1" s="4"/>
       <c r="D1" s="4"/>
       <c r="E1" s="4"/>
@@ -2952,11 +3171,12 @@
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="B1:H1"/>
     <mergeCell ref="A2:H2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -2971,11 +3191,10 @@
     <col min="4" max="5" width="16" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="36" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1" s="4" t="s">
+    <row r="1" ht="40" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B1" s="4" t="s">
         <v>114</v>
       </c>
-      <c r="B1" s="4"/>
       <c r="C1" s="4"/>
       <c r="D1" s="4"/>
       <c r="E1" s="4"/>
@@ -3264,11 +3483,12 @@
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="B1:H1"/>
     <mergeCell ref="A2:H2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -3287,11 +3507,10 @@
     <col min="9" max="9" width="30" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="36" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1" s="4" t="s">
+    <row r="1" ht="40" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B1" s="4" t="s">
         <v>152</v>
       </c>
-      <c r="B1" s="4"/>
       <c r="C1" s="4"/>
       <c r="D1" s="4"/>
       <c r="E1" s="4"/>
@@ -3818,7 +4037,7 @@
     <row r="300" spans="7:8" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="B1:H1"/>
     <mergeCell ref="A2:H2"/>
   </mergeCells>
   <dataValidations count="4">
@@ -3837,5 +4056,6 @@
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Fix spreadsheet logo: pure black cat, larger size
</commit_message>
<xml_diff>
--- a/downloads/blackcat-airbnb-profit-tracker.xlsx
+++ b/downloads/blackcat-airbnb-profit-tracker.xlsx
@@ -817,7 +817,7 @@
       <xdr:row>0</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="304800" cy="304800"/>
+    <xdr:ext cx="419100" cy="419100"/>
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="1" name="Picture 1">
@@ -861,7 +861,7 @@
       <xdr:row>0</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="304800" cy="304800"/>
+    <xdr:ext cx="419100" cy="419100"/>
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="1" name="Picture 1">
@@ -905,7 +905,7 @@
       <xdr:row>0</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="304800" cy="304800"/>
+    <xdr:ext cx="419100" cy="419100"/>
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="1" name="Picture 1">
@@ -949,7 +949,7 @@
       <xdr:row>0</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="304800" cy="304800"/>
+    <xdr:ext cx="419100" cy="419100"/>
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="1" name="Picture 1">
@@ -993,7 +993,7 @@
       <xdr:row>0</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="304800" cy="304800"/>
+    <xdr:ext cx="419100" cy="419100"/>
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="1" name="Picture 1">
@@ -1557,7 +1557,7 @@
     <col min="8" max="8" width="30" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="40" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="1" ht="48" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B1" s="4" t="s">
         <v>32</v>
       </c>
@@ -2669,7 +2669,7 @@
     <col min="14" max="14" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="40" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="1" ht="48" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B1" s="4" t="s">
         <v>85</v>
       </c>
@@ -3025,7 +3025,7 @@
     <col min="8" max="8" width="22" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="40" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="1" ht="48" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B1" s="4" t="s">
         <v>107</v>
       </c>
@@ -3191,7 +3191,7 @@
     <col min="4" max="5" width="16" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="40" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="1" ht="48" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B1" s="4" t="s">
         <v>114</v>
       </c>
@@ -3507,7 +3507,7 @@
     <col min="9" max="9" width="30" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="40" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="1" ht="48" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B1" s="4" t="s">
         <v>152</v>
       </c>

</xml_diff>

<commit_message>
Regenerate profit-tracker spreadsheet from updated source
The shipped .xlsx predated two source changes to generate-spreadsheet.js:
the UTM-tagged signup link (utm_medium=spreadsheet) and the 15.5%
host-fee transition note on the sample fee rows. Rebuilt with the app
repo's exceljs; verified the tagged link and fee note are present in
the output. First tracked file_download landed this week — future
downloaders now carry attribution.
</commit_message>
<xml_diff>
--- a/downloads/blackcat-airbnb-profit-tracker.xlsx
+++ b/downloads/blackcat-airbnb-profit-tracker.xlsx
@@ -108,7 +108,7 @@
     <t>generates tax reports, and gives you AI-powered insights.</t>
   </si>
   <si>
-    <t>→ https://app.tryblackcat.com/signup (Free to start)</t>
+    <t>→ https://app.tryblackcat.com/signup?utm_source=tryblackcat&amp;utm_medium=spreadsheet&amp;utm_content=xlsx_instructions (Free to start)</t>
   </si>
   <si>
     <t>Questions? support@tryblackcat.com</t>
@@ -270,7 +270,7 @@
     <t>Airbnb host fee — January</t>
   </si>
   <si>
-    <t>3% of gross</t>
+    <t>3% of gross (15.5% from Sept 15, 2026)</t>
   </si>
   <si>
     <t>Black Cat Analytics — Monthly Dashboard</t>

</xml_diff>